<commit_message>
docs(grille): MAJ competences RGPD/SEO apres consentement + PostHog EU
Grille d'evaluation RNCP remise a jour suite au chantier consentement + PostHog EU
(retrait Umami). Corrige des references devenues obsoletes et renforce la preuve :

- C11 (R39, RGPD) : la preuve fil rouge cite desormais le VRAI outil de
  consentement a categories (cookie-consent.tsx + CookieConsent.tsx landing,
  PostHog en opt-in, revocable) au lieu de l'ancien cookie-banner.tsx (supprime).
  Statut inchange (« a detailler ») : dependance au cas externe E9 preservee.
- C20 (R79) : outil d'audience = PostHog EU (consentement) au lieu d'Umami.
- C20 (R80) : integration verifiee = ilot PostHog gate + dashboard, au lieu de
  AudienceTracking.astro (supprime).
- C3 (R14) : registre = 9 traitements (au lieu de 8).

Seules les chaines concernees sont modifiees ; mise en forme preservee.
Original recuperable via l'historique git.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/memoire/Grille_evaluation_TaskForce_REMPLIE_DFS_25-26.xlsx
+++ b/memoire/Grille_evaluation_TaskForce_REMPLIE_DFS_25-26.xlsx
@@ -98,7 +98,7 @@
     <t>Le projet est en adéquation avec le cadre réglementaire et législatif, il anticipe le cas échéant l’évolution connue des normes.</t>
   </si>
   <si>
-    <t>Abordé. Conformité RGPD traitée : registre des traitements Art. 30 (8 traitements, bases légales, sous-traitants), audit de conformité, droits des personnes implémentés (export et effacement via GdprService), double opt-in à l'inscription, et durées de conservation appliquées automatiquement depuis le 23/07 (RetentionScheduler).</t>
+    <t>Abordé. Conformité RGPD traitée : registre des traitements Art. 30 (9 traitements, bases légales, sous-traitants), audit de conformité, droits des personnes implémentés (export et effacement via GdprService), double opt-in à l'inscription, et durées de conservation appliquées automatiquement depuis le 23/07 (RetentionScheduler).</t>
   </si>
   <si>
     <t>Les possibilités d’aménagement inclusif et d’écoconception sont analysées et prises en considération.</t>
@@ -266,7 +266,7 @@
     <t>-      Un outil de recueil du consentement de l’utilisateur vis-à-vis des cookies est proposé pour implémentation, ses caractéristiques techniques sont détaillées,</t>
   </si>
   <si>
-    <t>Traite sur le projet fil rouge, a defaut du cas externe. Le referentiel (p. 8) rattache ce critere au livrable E9, un audit RGPD d'un site marchand existant FOURNI par le certificateur, hors projet fil rouge. Ce sujet n'a pas ete communique a ce jour ; il a ete reclame. En l'absence de support impose, l'audit a ete conduit sur TaskForce (`Audit_RGPD_Conformite.md`), ce qui demontre la meme competence technique. A refaire sur le site fourni s'il est transmis. Preuve sur le fil rouge : banniere de consentement implementee (`frontend/components/common/cookie-banner.tsx`, montee dans `app/layout.tsx`), caracteristiques techniques documentees dans `Politique_Confidentialite_CGU.md`.</t>
+    <t xml:space="preserve">Traite sur le projet fil rouge, a defaut du cas externe. Le referentiel (p. 8) rattache ce critere au livrable E9, un audit RGPD d'un site marchand existant FOURNI par le certificateur, hors projet fil rouge. Ce sujet n'a pas ete communique a ce jour ; il a ete reclame. En l'absence de support impose, l'audit a ete conduit sur TaskForce (`Audit_RGPD_Conformite.md`), ce qui demontre la meme competence technique. A refaire sur le site fourni s'il est transmis. Preuve sur le fil rouge : VERITABLE outil de recueil du consentement a categories deploye (app `frontend/components/common/cookie-consent.tsx` + landing `landing-page/src/components/site/CookieConsent.tsx`, montes au layout) : cookies necessaires exemptes + analytics (PostHog EU) en opt-in explicite, refusables et revocables a tout moment via « Manage cookies », aucun traceur avant consentement ; caracteristiques techniques detaillees dans `Politique_Confidentialite_CGU.md` et l'audit RGPD (traitement n°9).</t>
   </si>
   <si>
     <t>-      Une vue « politique de confidentialité et traitement des données à caractère personnel » est prévue.</t>
@@ -497,13 +497,13 @@
     <t>-      - Le choix des outils de mesure d’audience et de performance marketing est pertinent : les outils sont les plus performants possibles au regard du besoin et des moyens du client.</t>
   </si>
   <si>
-    <t>Abordé. Outil retenu : Umami, auto-hébergé (`docker-compose.dev.yml` et `.prod.yml`). Le choix est motivé par la conformité et non par le confort : aucun cookie déposé, donc aucun consentement à recueillir, et aucun transfert hors UE, donc aucun destinataire étranger au registre des traitements. Une solution hébergée outre-Atlantique aurait contredit le retrait du fournisseur d'IA américain du 16/07 et l'auto-hébergement du modèle de langage. Mesures collectées : pages consultées, provenance, appareil, navigateur.</t>
+    <t xml:space="preserve">Abordé. Outil retenu : PostHog en offre EU Cloud (`eu.i.posthog.com`, projet dédié), chargé UNIQUEMENT après consentement (opt-in cookies). Le choix privilégie une vraie analyse produit tout en gardant les données dans l'UE (aucun transfert hors UE, cohérent avec le retrait du fournisseur d'IA américain et l'auto-hébergement du modèle). L'ancien plan Umami cookieless (exempté de consentement) a été retiré : PostHog dépose des identifiants et impose donc un consentement préalable, recueilli par un bandeau à catégories (nécessaires + analytics en opt-in). Mesures collectées après opt-in : pages consultées, provenance, appareil, navigateur, pays.</t>
   </si>
   <si>
     <t>-      L’intégration des outils de mesure de performance marketing est fonctionnelle.</t>
   </si>
   <si>
-    <t>Abordé. Intégration vérifiée de bout en bout le 23/07/2026 : le service répond, sert son script de mesure, et un événement de page émis vers l'API a été retrouvé en base avec sa provenance, son navigateur et son type d'appareil. Le script est injecté sur les 16 pages via un composant unique (`AudienceTracking.astro`), et n'est émis que si les variables d'environnement sont renseignées, afin que les constructions locales et les audits Lighthouse ne polluent pas les statistiques.</t>
+    <t xml:space="preserve">Abordé. Intégration PostHog vérifiée en direct : rien n'est chargé avant consentement (aucun cookie ni entrée localStorage `ph_`), et après opt-in l'initialisation part vers l'UE (`eu.i.posthog.com`, configuration distante récupérée) avec capture des pages vues, puis coupure (opt-out) à la révocation. Chargée sur toute la landing via un îlot unique (`CookieConsent.tsx`, `client:load`) et sur l'application (`posthog-provider.tsx`), toujours derrière le consentement. Un tableau de bord d'audience est configuré côté PostHog EU (pages vues, visiteurs uniques, sources, appareils, pays).</t>
   </si>
   <si>
     <t>-      L’application est conforme à au moins 70% des critères d’optimisation technique SEO en vigueur.</t>

</xml_diff>